<commit_message>
M9.0: pair-1 fixtures in the REAL sheet / document shape
STTM: meta r1-r10 (TBD / .dat / blanks, no Load Strategy row), bands
A14:I14, K14:P14, R14:W14, Y14:AD14, 27 headers over 30 columns (J / Q / X
empty), schema + table constants on every data row, Header / Details /
Trailer banner rows, one "Do Not Map" row without a data type.
FRD: Target Table Name = inline layer block, Target Catalog and Schema
blank, Object Name = "<label>: <file>" lines (names no feed), Name = a
sentence. Values stay the aliased golden's; the FAQ fixture follows the
derived feed id (vnd_p_accum_client).

Source: the two captures on acfc-hotfix-1 (not merged); scrubbed record in
docs/acfc/M9_FINDINGS.md. Commits M9.0-M9.4 are split by path and green
together (suite run on the M9.5 tree), not one by one.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/acfc_shapes/sttm/pair_1_family_a.xlsx
+++ b/fixtures/acfc_shapes/sttm/pair_1_family_a.xlsx
@@ -954,7 +954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA41"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -965,7 +965,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>I_ACCUM_*_TO_CLIENT_*.csv; I_ACCUM_*_FROM_CLIENT_*.csv; F_ACCUM_*_TO_CLIENT_*.csv; F_ACCUM_*_FROM_CLIENT_*.csv</t>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -977,7 +977,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>I_ACCUM_20260115_TO_CLIENT_0900.csv</t>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fixed Width Text</t>
+          <t>.dat</t>
         </is>
       </c>
     </row>
@@ -1057,42 +1057,23 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Load Strategy</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Append</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
           <t>Source Data</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Data Rules and Primary Keys</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>Staging Layer Table</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>Standard Layer Table</t>
         </is>
@@ -1144,270 +1125,148 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Data Definition</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>PII</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Primary Key</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Critical Data</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>Not NULL</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Load Rules</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>Workspace</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>Target Catalog</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>Target Schema Name in DL</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>Target Table Name in DL</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>Target_Column_Name_in_DL</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>Target Data Type in DL</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>Workspace</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t>Target Catalog</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="AA15" t="inlineStr">
         <is>
           <t>Target Schema Name in DL</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="AB15" t="inlineStr">
         <is>
           <t>Target Table Name in DL</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr">
+      <c r="AC15" t="inlineStr">
         <is>
           <t>Target_Column_Name_in_DL</t>
         </is>
       </c>
-      <c r="AA15" t="inlineStr">
+      <c r="AD15" t="inlineStr">
         <is>
           <t>Target Data Type in DL</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>HDDR</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>SEGMENT_IDENTIFIER</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H16" t="n">
-        <v>2</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Load as is</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>pr_dlk_vnd_p</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>stg_vnd_p_accum</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>SEGMENT_IDENTIFIER</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>pr_std_vnd_p</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>accum</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>SEGMENT_IDENTIFIER</t>
-        </is>
-      </c>
-      <c r="AA16" t="inlineStr">
-        <is>
-          <t>String</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Header</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HDDR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SEGMENT_IDENTIFIER</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
         <v>2</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>HDDR</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>FILE_TYPE</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>3</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1</v>
-      </c>
       <c r="H17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>File type indicator</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>File type indicator</t>
+          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
+          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1419,65 +1278,70 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>FILE_TYPE</t>
-        </is>
-      </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>SEGMENT_IDENTIFIER</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="AA17" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z17" t="inlineStr">
-        <is>
-          <t>FILE_TYPE</t>
-        </is>
-      </c>
-      <c r="AA17" t="inlineStr">
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>SEGMENT_IDENTIFIER</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
         <is>
           <t>String</t>
         </is>
@@ -1485,53 +1349,48 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HDDR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>FILE_TYPE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>3</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>HDDR</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>DATA_CATEGORY</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>4</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Data category indicator</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Data category indicator</t>
+          <t>File type indicator</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
+          <t>File type indicator</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1543,65 +1402,70 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>DATA_CATEGORY</t>
-        </is>
-      </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>FILE_TYPE</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
+      <c r="AA18" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t>DATA_CATEGORY</t>
-        </is>
-      </c>
-      <c r="AA18" t="inlineStr">
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>FILE_TYPE</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
         <is>
           <t>String</t>
         </is>
@@ -1609,177 +1473,172 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HDDR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DATA_CATEGORY</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
         <v>4</v>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>HDDR</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>PROCESS_DATE</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>5</v>
-      </c>
       <c r="G19" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>File process date (yyyyMMdd)</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>File process date (yyyyMMdd)</t>
+          <t>Data category indicator</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
+          <t>Data category indicator</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Convert yyyyMMdd to yyyy-MM-dd</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
+          <t>Load as is</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>PROCESS_DATE</t>
-        </is>
-      </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>DATA_CATEGORY</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
+      <c r="AA19" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>PROCESS_DATE</t>
-        </is>
-      </c>
-      <c r="AA19" t="inlineStr">
-        <is>
-          <t>Date</t>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>DATA_CATEGORY</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>String</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HDDR</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PROCESS_DATE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
         <v>5</v>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>HDDR</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>PROCESS_TIME</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>13</v>
-      </c>
       <c r="G20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H20" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>File process time (HHmmss)</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>File process time (HHmmss)</t>
+          <t>File process date (yyyyMMdd)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
+          <t>File process date (yyyyMMdd)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1791,119 +1650,119 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Load as is</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
+          <t>Convert yyyyMMdd to yyyy-MM-dd</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>PROCESS_TIME</t>
-        </is>
-      </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>PROCESS_DATE</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
+      <c r="AA20" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>PROCESS_TIME</t>
-        </is>
-      </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>String</t>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>PROCESS_DATE</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Date</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HDDR</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PROCESS_TIME</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>13</v>
+      </c>
+      <c r="G21" t="n">
         <v>6</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>HDDR</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>GROUP_ID</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>19</v>
-      </c>
-      <c r="G21" t="n">
-        <v>10</v>
-      </c>
       <c r="H21" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Group identifier</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Group identifier</t>
+          <t>File process time (HHmmss)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
+          <t>File process time (HHmmss)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1915,65 +1774,70 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>GROUP_ID</t>
-        </is>
-      </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>PROCESS_TIME</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
+      <c r="AA21" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z21" t="inlineStr">
-        <is>
-          <t>GROUP_ID</t>
-        </is>
-      </c>
-      <c r="AA21" t="inlineStr">
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>PROCESS_TIME</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
         <is>
           <t>String</t>
         </is>
@@ -1981,7 +1845,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1990,7 +1854,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FILLER_1</t>
+          <t>GROUP_ID</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2004,30 +1868,25 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="G22" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H22" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Filler</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Filler</t>
+          <t>Group identifier</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
+          <t>Group identifier</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2039,65 +1898,70 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>FILLER_1</t>
-        </is>
-      </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>GROUP_ID</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
+      <c r="AA22" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z22" t="inlineStr">
-        <is>
-          <t>FILLER_1</t>
-        </is>
-      </c>
-      <c r="AA22" t="inlineStr">
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>GROUP_ID</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
         <is>
           <t>String</t>
         </is>
@@ -2105,7 +1969,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2114,7 +1978,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>VERSION_RELEASE</t>
+          <t>FILLER_1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2128,30 +1992,25 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H23" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Layout version/release</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Layout version/release</t>
+          <t>Filler</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
+          <t>Filler</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2163,65 +2022,70 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>VERSION_RELEASE</t>
-        </is>
-      </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>FILLER_1</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
+      <c r="AA23" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>VERSION_RELEASE</t>
-        </is>
-      </c>
-      <c r="AA23" t="inlineStr">
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>FILLER_1</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
         <is>
           <t>String</t>
         </is>
@@ -2229,21 +2093,21 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>HDDR</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SEGMENT_IDENTIFIER</t>
+          <t>VERSION_RELEASE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2252,232 +2116,115 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="G24" t="n">
         <v>2</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
+          <t>Layout version/release</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
+          <t>Layout version/release</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>SEGMENT_IDENTIFIER</t>
-        </is>
-      </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>VERSION_RELEASE</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="AA24" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z24" t="inlineStr">
-        <is>
-          <t>SEGMENT_IDENTIFIER</t>
-        </is>
-      </c>
-      <c r="AA24" t="inlineStr">
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>VERSION_RELEASE</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>10</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>DET</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>CARDHOLDER_ID</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>3</v>
-      </c>
-      <c r="G25" t="n">
-        <v>15</v>
-      </c>
-      <c r="H25" t="n">
-        <v>17</v>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Cardholder identifier</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Cardholder identifier</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Load as is</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>pr_dlk_vnd_p</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>stg_vnd_p_accum</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>CARDHOLDER_ID</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t>pr_std_vnd_p</t>
-        </is>
-      </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>accum</t>
-        </is>
-      </c>
-      <c r="Y25" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z25" t="inlineStr">
-        <is>
-          <t>CARDHOLDER_ID</t>
-        </is>
-      </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>String</t>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Details</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2486,7 +2233,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PLAN_ID</t>
+          <t>SEGMENT_IDENTIFIER</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2500,100 +2247,100 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Plan identifier</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Plan identifier</t>
+          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
+          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="T26" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>PLAN_ID</t>
-        </is>
-      </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>SEGMENT_IDENTIFIER</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="AA26" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z26" t="inlineStr">
-        <is>
-          <t>PLAN_ID</t>
-        </is>
-      </c>
-      <c r="AA26" t="inlineStr">
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>SEGMENT_IDENTIFIER</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
         <is>
           <t>String</t>
         </is>
@@ -2601,7 +2348,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2610,12 +2357,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>INDIVIDUAL_DEDUCTIBLE</t>
+          <t>CARDHOLDER_ID</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2624,30 +2371,25 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="G27" t="n">
+        <v>15</v>
+      </c>
+      <c r="H27" t="n">
         <v>17</v>
       </c>
-      <c r="H27" t="n">
-        <v>50</v>
-      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Individual deductible accumulated amount</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Individual deductible accumulated amount</t>
+          <t>Cardholder identifier</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
+          <t>Cardholder identifier</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2659,73 +2401,78 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="T27" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>INDIVIDUAL_DEDUCTIBLE</t>
-        </is>
-      </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Decimal(17,2)</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>CARDHOLDER_ID</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
+      <c r="AA27" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z27" t="inlineStr">
-        <is>
-          <t>INDIVIDUAL_DEDUCTIBLE</t>
-        </is>
-      </c>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>Decimal(17,2)</t>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>CARDHOLDER_ID</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>String</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2734,12 +2481,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FAMILY_DEDUCTIBLE</t>
+          <t>PLAN_ID</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2748,30 +2495,25 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="G28" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H28" t="n">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Family deductible accumulated amount</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Family deductible accumulated amount</t>
+          <t>Plan identifier</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
+          <t>Plan identifier</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2783,73 +2525,78 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="T28" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>FAMILY_DEDUCTIBLE</t>
-        </is>
-      </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Decimal(18,2)</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>PLAN_ID</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
+      <c r="AA28" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z28" t="inlineStr">
-        <is>
-          <t>FAMILY_DEDUCTIBLE</t>
-        </is>
-      </c>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>Decimal(18,2)</t>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>PLAN_ID</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>String</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2858,7 +2605,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COPAY</t>
+          <t>INDIVIDUAL_DEDUCTIBLE</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2872,30 +2619,25 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="G29" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H29" t="n">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Copay accumulated amount</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Copay accumulated amount</t>
+          <t>Individual deductible accumulated amount</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
+          <t>Individual deductible accumulated amount</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2907,73 +2649,78 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>COPAY</t>
-        </is>
-      </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Decimal(19,2)</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>INDIVIDUAL_DEDUCTIBLE</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
+          <t>Decimal(17,2)</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="AA29" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z29" t="inlineStr">
-        <is>
-          <t>COPAY</t>
-        </is>
-      </c>
-      <c r="AA29" t="inlineStr">
-        <is>
-          <t>Decimal(19,2)</t>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>INDIVIDUAL_DEDUCTIBLE</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>Decimal(17,2)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2982,7 +2729,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COINSURANCE</t>
+          <t>FAMILY_DEDUCTIBLE</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2996,30 +2743,25 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="G30" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H30" t="n">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Coinsurance accumulated amount</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Coinsurance accumulated amount</t>
+          <t>Family deductible accumulated amount</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
+          <t>Family deductible accumulated amount</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3031,73 +2773,78 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="T30" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>COINSURANCE</t>
-        </is>
-      </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Decimal(20,2)</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>FAMILY_DEDUCTIBLE</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
+          <t>Decimal(18,2)</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
+      <c r="AA30" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z30" t="inlineStr">
-        <is>
-          <t>COINSURANCE</t>
-        </is>
-      </c>
-      <c r="AA30" t="inlineStr">
-        <is>
-          <t>Decimal(20,2)</t>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>FAMILY_DEDUCTIBLE</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>Decimal(18,2)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -3106,7 +2853,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>INDIVIDUAL_LIMIT</t>
+          <t>COPAY</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3120,30 +2867,25 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>108</v>
+        <v>69</v>
       </c>
       <c r="G31" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H31" t="n">
-        <v>128</v>
+        <v>87</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Individual out-of-pocket limit</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Individual out-of-pocket limit</t>
+          <t>Copay accumulated amount</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
+          <t>Copay accumulated amount</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3155,73 +2897,78 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="T31" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>INDIVIDUAL_LIMIT</t>
-        </is>
-      </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Decimal(21,2)</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>COPAY</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
+          <t>Decimal(19,2)</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr">
+      <c r="AA31" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z31" t="inlineStr">
-        <is>
-          <t>INDIVIDUAL_LIMIT</t>
-        </is>
-      </c>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>Decimal(21,2)</t>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>COPAY</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>Decimal(19,2)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -3230,7 +2977,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FAMILY_LIMIT</t>
+          <t>COINSURANCE</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3244,30 +2991,25 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>129</v>
+        <v>88</v>
       </c>
       <c r="G32" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H32" t="n">
-        <v>150</v>
+        <v>107</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Family out-of-pocket limit</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Family out-of-pocket limit</t>
+          <t>Coinsurance accumulated amount</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
+          <t>Coinsurance accumulated amount</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3279,73 +3021,78 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
+      <c r="T32" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>FAMILY_LIMIT</t>
-        </is>
-      </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Decimal(22,2)</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>COINSURANCE</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
+          <t>Decimal(20,2)</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr">
+      <c r="AA32" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y32" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z32" t="inlineStr">
-        <is>
-          <t>FAMILY_LIMIT</t>
-        </is>
-      </c>
-      <c r="AA32" t="inlineStr">
-        <is>
-          <t>Decimal(22,2)</t>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>COINSURANCE</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>Decimal(20,2)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -3354,7 +3101,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PLAN_YEAR_START_DATE</t>
+          <t>INDIVIDUAL_LIMIT</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3368,30 +3115,25 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>151</v>
+        <v>108</v>
       </c>
       <c r="G33" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H33" t="n">
-        <v>173</v>
+        <v>128</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Plan year start date (yyyyMMdd)</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Plan year start date (yyyyMMdd)</t>
+          <t>Individual out-of-pocket limit</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
+          <t>Individual out-of-pocket limit</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3403,73 +3145,78 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Convert yyyyMMdd to yyyy-MM-dd</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
+          <t>Load as is</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
+      <c r="T33" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>PLAN_YEAR_START_DATE</t>
-        </is>
-      </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>INDIVIDUAL_LIMIT</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
+          <t>Decimal(21,2)</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr">
+      <c r="AA33" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y33" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z33" t="inlineStr">
-        <is>
-          <t>PLAN_YEAR_START_DATE</t>
-        </is>
-      </c>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>Date</t>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>INDIVIDUAL_LIMIT</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>Decimal(21,2)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -3478,7 +3225,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PLAN_YEAR_END_DATE</t>
+          <t>FAMILY_LIMIT</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3492,30 +3239,25 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>174</v>
+        <v>129</v>
       </c>
       <c r="G34" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H34" t="n">
-        <v>197</v>
+        <v>150</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Plan year end date (yyyyMMdd)</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Plan year end date (yyyyMMdd)</t>
+          <t>Family out-of-pocket limit</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
+          <t>Family out-of-pocket limit</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3527,73 +3269,78 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Convert yyyyMMdd to yyyy-MM-dd</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
+          <t>Load as is</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
+      <c r="T34" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>PLAN_YEAR_END_DATE</t>
-        </is>
-      </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>FAMILY_LIMIT</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
+          <t>Decimal(22,2)</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr">
+      <c r="AA34" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y34" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z34" t="inlineStr">
-        <is>
-          <t>PLAN_YEAR_END_DATE</t>
-        </is>
-      </c>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>Date</t>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>FAMILY_LIMIT</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>Decimal(22,2)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -3602,7 +3349,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FILLER_2</t>
+          <t>PLAN_YEAR_START_DATE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3616,30 +3363,25 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>198</v>
+        <v>151</v>
       </c>
       <c r="G35" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H35" t="n">
-        <v>222</v>
+        <v>173</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Filler</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Filler</t>
+          <t>Plan year start date (yyyyMMdd)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
+          <t>Plan year start date (yyyyMMdd)</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3651,87 +3393,92 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Load as is</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
+          <t>Convert yyyyMMdd to yyyy-MM-dd</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr">
+      <c r="T35" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>FILLER_2</t>
-        </is>
-      </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>PLAN_YEAR_START_DATE</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr">
+      <c r="AA35" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y35" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z35" t="inlineStr">
-        <is>
-          <t>FILLER_2</t>
-        </is>
-      </c>
-      <c r="AA35" t="inlineStr">
-        <is>
-          <t>String</t>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>PLAN_YEAR_START_DATE</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>Date</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TRLR</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SEGMENT_IDENTIFIER</t>
+          <t>PLAN_YEAR_END_DATE</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3740,122 +3487,122 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>174</v>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="H36" t="n">
-        <v>2</v>
+        <v>197</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
+          <t>Plan year end date (yyyyMMdd)</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
+          <t>Plan year end date (yyyyMMdd)</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Load as is</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
+          <t>Convert yyyyMMdd to yyyy-MM-dd</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="T36" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>SEGMENT_IDENTIFIER</t>
-        </is>
-      </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>PLAN_YEAR_END_DATE</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr">
+      <c r="AA36" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y36" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z36" t="inlineStr">
-        <is>
-          <t>SEGMENT_IDENTIFIER</t>
-        </is>
-      </c>
-      <c r="AA36" t="inlineStr">
-        <is>
-          <t>String</t>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>PLAN_YEAR_END_DATE</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>Date</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TRLR</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LINE_COUNT</t>
+          <t>FILLER_2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3864,100 +3611,100 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3</v>
+        <v>198</v>
       </c>
       <c r="G37" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H37" t="n">
-        <v>12</v>
+        <v>222</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Number of detail records in the file</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Number of detail records in the file</t>
+          <t>Filler</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
+          <t>Filler</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>LINE_COUNT</t>
-        </is>
-      </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>vnd_p_accum_client</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>DLK</t>
+          <t>FILLER_2</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr">
+      <c r="AA37" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z37" t="inlineStr">
-        <is>
-          <t>LINE_COUNT</t>
-        </is>
-      </c>
-      <c r="AA37" t="inlineStr">
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>FILLER_2</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
         <is>
           <t>String</t>
         </is>
@@ -3965,339 +3712,704 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
+        <v>21</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Reserved Group
+(01)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>223</v>
+      </c>
+      <c r="G38" t="n">
+        <v>10</v>
+      </c>
+      <c r="H38" t="n">
+        <v>232</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Reserved for future use</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Reserved for future use</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>pr_dlk_vnd_p</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>stg_vnd_p_accum</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Do Not Map</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>pr_std_vnd_p</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>accum</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>Do Not Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>22</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TRLR</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SEGMENT_IDENTIFIER</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>2</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Record segment marker: 00 header, 10 detail, 99 trailer</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Load as is</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>pr_dlk_vnd_p</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>stg_vnd_p_accum</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>SEGMENT_IDENTIFIER</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>pr_std_vnd_p</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>accum</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>SEGMENT_IDENTIFIER</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
         <v>23</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>TRLR</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>LINE_COUNT</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" t="n">
+        <v>10</v>
+      </c>
+      <c r="H41" t="n">
+        <v>12</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Number of detail records in the file</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Number of detail records in the file</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Load as is</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>pr_dlk_vnd_p</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>stg_vnd_p_accum</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>LINE_COUNT</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>pr_std_vnd_p</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>accum</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>LINE_COUNT</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>24</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TRLR</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
         <is>
           <t>FILLER_3</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
         <v>13</v>
       </c>
-      <c r="G38" t="n">
+      <c r="G42" t="n">
         <v>20</v>
       </c>
-      <c r="H38" t="n">
+      <c r="H42" t="n">
         <v>32</v>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Filler</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>Filler</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
         <is>
           <t>Load as is</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr">
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
+      <c r="T42" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T38" t="inlineStr">
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
         <is>
           <t>FILLER_3</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="W38" t="inlineStr">
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
         <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr">
+      <c r="AA42" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y38" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z38" t="inlineStr">
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
         <is>
           <t>FILLER_3</t>
         </is>
       </c>
-      <c r="AA38" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="C39" t="inlineStr">
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Audit column</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
         <is>
           <t>SRC_FILE_NAME</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="W43" t="inlineStr">
         <is>
           <t>STRING</t>
         </is>
       </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="W39" t="inlineStr">
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
         <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr">
+      <c r="AA43" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z39" t="inlineStr">
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr">
         <is>
           <t>SRC_FILE_NAME</t>
         </is>
       </c>
-      <c r="AA39" t="inlineStr">
+      <c r="AD43" t="inlineStr">
         <is>
           <t>STRING</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="C40" t="inlineStr">
+    <row r="44">
+      <c r="C44" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>Audit column</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
+      <c r="T44" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr">
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
         <is>
           <t>REC_CREATION_TIME</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="W44" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="W40" t="inlineStr">
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
         <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr">
+      <c r="AA44" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y40" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z40" t="inlineStr">
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr">
         <is>
           <t>REC_CREATION_TIME</t>
         </is>
       </c>
-      <c r="AA40" t="inlineStr">
+      <c r="AD44" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="C41" t="inlineStr">
+    <row r="45">
+      <c r="C45" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>Audit column</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
         <is>
           <t>pr_dlk_vnd_p</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
+      <c r="T45" t="inlineStr">
         <is>
           <t>stg_vnd_p_accum</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="T41" t="inlineStr">
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
         <is>
           <t>REC_UPDATED_TIME</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="W45" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>DLK</t>
-        </is>
-      </c>
-      <c r="W41" t="inlineStr">
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>DLK</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
         <is>
           <t>pr_std_vnd_p</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
+      <c r="AA45" t="inlineStr">
         <is>
           <t>accum</t>
         </is>
       </c>
-      <c r="Y41" t="inlineStr">
-        <is>
-          <t>vnd_p_accum_client</t>
-        </is>
-      </c>
-      <c r="Z41" t="inlineStr">
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>vnd_p_accum_client</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr">
         <is>
           <t>REC_UPDATED_TIME</t>
         </is>
       </c>
-      <c r="AA41" t="inlineStr">
+      <c r="AD45" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
@@ -4305,9 +4417,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="P14:U14"/>
-    <mergeCell ref="J14:O14"/>
-    <mergeCell ref="V14:AA14"/>
+    <mergeCell ref="K14:P14"/>
+    <mergeCell ref="Y14:AD14"/>
+    <mergeCell ref="R14:W14"/>
     <mergeCell ref="A14:I14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
M9.1b (1/4): Object Name as a block; pair-1 fixtures in the real-run shapes
The real Object Name cell (acfc-runs: PAIR1_REAL_RUN.md) is stanzas — a
"<line of business>:" line, the file pattern on the NEXT line; v0.5.1 read only
"<label>: <file>" on one line, so the FRD yielded no pattern. A multi-line
block or a nested label | value table is now read per line / row: feed name
from a feed-name label's value, files from a File-Name-type label or any
file-like value under another label; unlabelled values are never taken.
Fixture: the stanza cell; STTM meta rows 11-12 restored (Load Strategy =
Append, Notes) — the first capture stopped at r10.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/acfc_shapes/sttm/pair_1_family_a.xlsx
+++ b/fixtures/acfc_shapes/sttm/pair_1_family_a.xlsx
@@ -1057,6 +1057,25 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Load Strategy</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Append</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>

</xml_diff>